<commit_message>
20260518 next steps for assignment
</commit_message>
<xml_diff>
--- a/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
+++ b/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F19"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,6 +451,16 @@
           <t>uname_mgl</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>val_mol_l</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>orchestra_param</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -479,6 +489,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G2" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Nikkel [Ni]</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -507,6 +525,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G3" t="n">
+        <v>370</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Chloride</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -535,6 +561,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G4" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Silicium [Si]</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -563,6 +597,14 @@
           <t>°C</t>
         </is>
       </c>
+      <c r="G5" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Temperatuur</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -591,6 +633,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G6" t="n">
+        <v>410</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Calcium [Ca]</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -619,6 +669,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G7" t="n">
+        <v>120</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Magnesium [Mg]</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -647,6 +705,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G8" t="n">
+        <v>0.029</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Arseen [As]</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -675,6 +741,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G9" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Zink [Zn]</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -703,6 +777,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G10" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Sulfide</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -731,6 +813,14 @@
           <t>-</t>
         </is>
       </c>
+      <c r="G11" t="n">
+        <v>7.16</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>pH</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -759,6 +849,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G12" t="n">
+        <v>200</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Kalium [K]</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -787,6 +885,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G13" t="n">
+        <v>372.3188405797102</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Ammonium (als NH4)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -815,6 +921,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G14" t="n">
+        <v>1</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Mangaan [Mn]</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -843,6 +957,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G15" t="n">
+        <v>2600</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>Bicarbonaat</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -871,6 +993,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G16" t="n">
+        <v>400</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>Natrium [Na]</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -899,6 +1029,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G17" t="n">
+        <v>7.492613159424033</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Fosfaat (als PO4)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -927,6 +1065,14 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G18" t="n">
+        <v>769.6257018091079</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Sulfaat (als SO4)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -955,6 +1101,62 @@
           <t>mg/l</t>
         </is>
       </c>
+      <c r="G19" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>IJzer [Fe]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr"/>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="n">
+        <v>3.52112676056338e-06</v>
+      </c>
+      <c r="H20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr"/>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="n">
+        <v>4.147145921217188e-08</v>
+      </c>
+      <c r="H21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr"/>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr"/>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="n">
+        <v>1.294256490952006e-07</v>
+      </c>
+      <c r="H22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr"/>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="n">
+        <v>5.960323814607242e-09</v>
+      </c>
+      <c r="H23" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
20260521 understood *.diss construct pyOrchestra
</commit_message>
<xml_diff>
--- a/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
+++ b/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
@@ -469,10 +469,10 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D2" t="n">
-        <v>410</v>
+        <v>0.87</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -480,11 +480,11 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.01022954091816367</v>
+        <v>1.583545686203131e-05</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ca+2.tot</t>
+          <t>Mn+2.tot</t>
         </is>
       </c>
     </row>
@@ -500,10 +500,10 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D3" t="n">
-        <v>400</v>
+        <v>1</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -511,11 +511,11 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.01739886907351022</v>
+        <v>1.790510295434199e-05</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Na+.tot</t>
+          <t>Fe+2.tot</t>
         </is>
       </c>
     </row>
@@ -531,10 +531,10 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>440</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -542,11 +542,11 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.005115089514066497</v>
+        <v>0.01913875598086125</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>K+.tot</t>
+          <t>Na+.tot</t>
         </is>
       </c>
     </row>
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D5" t="n">
-        <v>15.9</v>
+        <v>329.8627573300062</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -573,11 +573,11 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.0005660377358490566</v>
+        <v>0.003433924186237833</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Si.tot</t>
+          <t>SO4-2.tot</t>
         </is>
       </c>
     </row>
@@ -593,22 +593,22 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D6" t="n">
-        <v>370</v>
+        <v>7.13</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.01043723554301833</v>
+        <v>7.13</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Cl-.tot</t>
+          <t>pH</t>
         </is>
       </c>
     </row>
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D7" t="n">
-        <v>0.12</v>
+        <v>150.3734782608696</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -635,11 +635,11 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.741814780168382e-06</v>
+        <v>0.008335558661910733</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>S-2.tot</t>
+          <t>NH4+.tot</t>
         </is>
       </c>
     </row>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D8" t="n">
-        <v>4.2</v>
+        <v>0.1</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -666,11 +666,11 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7.520143240823636e-05</v>
+        <v>3.118178983473652e-06</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Fe+2.tot</t>
+          <t>S-2.tot</t>
         </is>
       </c>
     </row>
@@ -686,10 +686,10 @@
         </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D9" t="n">
-        <v>2600</v>
+        <v>21</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -697,11 +697,11 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.04260898066207801</v>
+        <v>0.0007475970096119616</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>HCO3-.tot</t>
+          <t>Si.tot</t>
         </is>
       </c>
     </row>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D10" t="n">
-        <v>7.492613159424033</v>
+        <v>460</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -728,11 +728,11 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>7.889452626538941e-05</v>
+        <v>0.01147704590818363</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>PO4-3.tot</t>
+          <t>Ca+2.tot</t>
         </is>
       </c>
     </row>
@@ -748,10 +748,10 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D11" t="n">
-        <v>769.6257018091079</v>
+        <v>507</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -759,11 +759,11 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.008011926939507683</v>
+        <v>0.01430183356840621</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>SO4-2.tot</t>
+          <t>Cl-.tot</t>
         </is>
       </c>
     </row>
@@ -779,10 +779,10 @@
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D12" t="n">
-        <v>120</v>
+        <v>11.25</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -790,11 +790,11 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.004936240230357877</v>
+        <v>0.0001184584605664947</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Mg+2.tot</t>
+          <t>PO4-3.tot</t>
         </is>
       </c>
     </row>
@@ -810,22 +810,22 @@
         </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D13" t="n">
-        <v>18.6</v>
+        <v>3800</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>mg/l</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>291.75</v>
+        <v>0.06227466404457555</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>HCO3-.tot</t>
         </is>
       </c>
     </row>
@@ -841,10 +841,10 @@
         </is>
       </c>
       <c r="C14" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>180</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -852,11 +852,11 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.820167455405897e-05</v>
+        <v>0.007404360345536817</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Mn+2.tot</t>
+          <t>Mg+2.tot</t>
         </is>
       </c>
     </row>
@@ -872,22 +872,22 @@
         </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D15" t="n">
-        <v>372.3188405797102</v>
+        <v>14.7</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.02063851666184647</v>
+        <v>287.85</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NH4+.tot</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -903,22 +903,22 @@
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>45272</v>
+        <v>46002</v>
       </c>
       <c r="D16" t="n">
-        <v>7.16</v>
+        <v>210</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mg/l</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>7.16</v>
+        <v>0.005370843989769821</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>K+.tot</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
20260522 finalized group assignment leachate
</commit_message>
<xml_diff>
--- a/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
+++ b/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
@@ -469,10 +469,10 @@
         </is>
       </c>
       <c r="C2" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D2" t="n">
-        <v>0.87</v>
+        <v>410</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
@@ -480,11 +480,11 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>1.583545686203131e-05</v>
+        <v>0.01022954091816367</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Mn+2.tot</t>
+          <t>Ca+2.tot</t>
         </is>
       </c>
     </row>
@@ -500,10 +500,10 @@
         </is>
       </c>
       <c r="C3" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D3" t="n">
-        <v>1</v>
+        <v>400</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -511,11 +511,11 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1.790510295434199e-05</v>
+        <v>0.01739886907351022</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Fe+2.tot</t>
+          <t>Na+.tot</t>
         </is>
       </c>
     </row>
@@ -531,10 +531,10 @@
         </is>
       </c>
       <c r="C4" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D4" t="n">
-        <v>440</v>
+        <v>200</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -542,11 +542,11 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.01913875598086125</v>
+        <v>0.005115089514066497</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Na+.tot</t>
+          <t>K+.tot</t>
         </is>
       </c>
     </row>
@@ -562,10 +562,10 @@
         </is>
       </c>
       <c r="C5" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D5" t="n">
-        <v>329.8627573300062</v>
+        <v>15.9</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -573,11 +573,11 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.003433924186237833</v>
+        <v>0.0005660377358490566</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>SO4-2.tot</t>
+          <t>Si.tot</t>
         </is>
       </c>
     </row>
@@ -593,22 +593,22 @@
         </is>
       </c>
       <c r="C6" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D6" t="n">
-        <v>7.13</v>
+        <v>370</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mg/l</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>7.13</v>
+        <v>0.01043723554301833</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>Cl-.tot</t>
         </is>
       </c>
     </row>
@@ -624,10 +624,10 @@
         </is>
       </c>
       <c r="C7" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D7" t="n">
-        <v>150.3734782608696</v>
+        <v>0.12</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -635,11 +635,11 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.008335558661910733</v>
+        <v>3.741814780168382e-06</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>NH4+.tot</t>
+          <t>S-2.tot</t>
         </is>
       </c>
     </row>
@@ -655,10 +655,10 @@
         </is>
       </c>
       <c r="C8" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D8" t="n">
-        <v>0.1</v>
+        <v>4.2</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -666,11 +666,11 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>3.118178983473652e-06</v>
+        <v>7.520143240823636e-05</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>S-2.tot</t>
+          <t>Fe+2.tot</t>
         </is>
       </c>
     </row>
@@ -686,10 +686,10 @@
         </is>
       </c>
       <c r="C9" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D9" t="n">
-        <v>21</v>
+        <v>2600</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -697,11 +697,11 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.0007475970096119616</v>
+        <v>0.04260898066207801</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Si.tot</t>
+          <t>HCO3-.tot</t>
         </is>
       </c>
     </row>
@@ -717,10 +717,10 @@
         </is>
       </c>
       <c r="C10" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D10" t="n">
-        <v>460</v>
+        <v>7.492613159424033</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -728,11 +728,11 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.01147704590818363</v>
+        <v>7.889452626538941e-05</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Ca+2.tot</t>
+          <t>PO4-3.tot</t>
         </is>
       </c>
     </row>
@@ -748,10 +748,10 @@
         </is>
       </c>
       <c r="C11" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D11" t="n">
-        <v>507</v>
+        <v>769.6257018091079</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -759,11 +759,11 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.01430183356840621</v>
+        <v>0.008011926939507683</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Cl-.tot</t>
+          <t>SO4-2.tot</t>
         </is>
       </c>
     </row>
@@ -779,10 +779,10 @@
         </is>
       </c>
       <c r="C12" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D12" t="n">
-        <v>11.25</v>
+        <v>120</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -790,11 +790,11 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.0001184584605664947</v>
+        <v>0.004936240230357877</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>PO4-3.tot</t>
+          <t>Mg+2.tot</t>
         </is>
       </c>
     </row>
@@ -810,22 +810,22 @@
         </is>
       </c>
       <c r="C13" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D13" t="n">
-        <v>3800</v>
+        <v>18.6</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>0.06227466404457555</v>
+        <v>291.75</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>HCO3-.tot</t>
+          <t>T</t>
         </is>
       </c>
     </row>
@@ -841,10 +841,10 @@
         </is>
       </c>
       <c r="C14" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D14" t="n">
-        <v>180</v>
+        <v>1</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -852,11 +852,11 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.007404360345536817</v>
+        <v>1.820167455405897e-05</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Mg+2.tot</t>
+          <t>Mn+2.tot</t>
         </is>
       </c>
     </row>
@@ -872,22 +872,22 @@
         </is>
       </c>
       <c r="C15" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D15" t="n">
-        <v>14.7</v>
+        <v>372.3188405797102</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>mg/l</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>287.85</v>
+        <v>0.02063851666184647</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>NH4+.tot</t>
         </is>
       </c>
     </row>
@@ -903,22 +903,22 @@
         </is>
       </c>
       <c r="C16" s="1" t="n">
-        <v>46002</v>
+        <v>45272</v>
       </c>
       <c r="D16" t="n">
-        <v>210</v>
+        <v>7.16</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.005370843989769821</v>
+        <v>7.16</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>K+.tot</t>
+          <t>pH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
20260527 started on violin plot for BB11Z
</commit_message>
<xml_diff>
--- a/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
+++ b/chemistry_book/content/project_THe/Orchestra_Project/tmp/df_work_PP-11N.xlsx
@@ -460,50 +460,50 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C2" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D2" t="n">
-        <v>410</v>
+        <v>6.81</v>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.01022954091816367</v>
+        <v>6.81</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Ca+2.tot</t>
+          <t>pH</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C3" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D3" t="n">
-        <v>400</v>
+        <v>60.68615692153924</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -511,30 +511,30 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.01739886907351022</v>
+        <v>0.003363977656404614</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Na+.tot</t>
+          <t>NH4+.tot</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C4" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D4" t="n">
-        <v>200</v>
+        <v>1415.281347473487</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
@@ -542,30 +542,30 @@
         </is>
       </c>
       <c r="F4" t="n">
-        <v>0.005115089514066497</v>
+        <v>0.01473330572010709</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>K+.tot</t>
+          <t>SO4-2.tot</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C5" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D5" t="n">
-        <v>15.9</v>
+        <v>290</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -573,30 +573,30 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.0005660377358490566</v>
+        <v>0.01261418007829491</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Si.tot</t>
+          <t>Na+.tot</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C6" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D6" t="n">
-        <v>370</v>
+        <v>130</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
@@ -604,30 +604,30 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.01043723554301833</v>
+        <v>0.003324808184143223</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Cl-.tot</t>
+          <t>K+.tot</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C7" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D7" t="n">
-        <v>0.12</v>
+        <v>650</v>
       </c>
       <c r="E7" t="inlineStr">
         <is>
@@ -635,30 +635,30 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3.741814780168382e-06</v>
+        <v>0.01621756487025948</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>S-2.tot</t>
+          <t>Ca+2.tot</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C8" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D8" t="n">
-        <v>4.2</v>
+        <v>170</v>
       </c>
       <c r="E8" t="inlineStr">
         <is>
@@ -666,30 +666,30 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7.520143240823636e-05</v>
+        <v>0.006993006993006994</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Fe+2.tot</t>
+          <t>Mg+2.tot</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C9" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D9" t="n">
-        <v>2600</v>
+        <v>1.2</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
@@ -697,30 +697,30 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.04260898066207801</v>
+        <v>2.184200946487077e-05</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>HCO3-.tot</t>
+          <t>Mn+2.tot</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C10" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D10" t="n">
-        <v>7.492613159424033</v>
+        <v>250</v>
       </c>
       <c r="E10" t="inlineStr">
         <is>
@@ -728,30 +728,30 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>7.889452626538941e-05</v>
+        <v>0.007052186177715091</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>PO4-3.tot</t>
+          <t>Cl-.tot</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C11" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D11" t="n">
-        <v>769.6257018091079</v>
+        <v>1600</v>
       </c>
       <c r="E11" t="inlineStr">
         <is>
@@ -759,30 +759,30 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.008011926939507683</v>
+        <v>0.02622091117666339</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>SO4-2.tot</t>
+          <t>HCO3-.tot</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C12" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D12" t="n">
-        <v>120</v>
+        <v>14.3</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
@@ -790,92 +790,92 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.004936240230357877</v>
+        <v>0.0005090779636881453</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Mg+2.tot</t>
+          <t>Si.tot</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C13" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D13" t="n">
-        <v>18.6</v>
+        <v>8.1</v>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>°C</t>
+          <t>mg/l</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>291.75</v>
+        <v>0.0001450313339301701</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>T</t>
+          <t>Fe+2.tot</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C14" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>13.3</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>mg/l</t>
+          <t>°C</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>1.820167455405897e-05</v>
+        <v>286.45</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Mn+2.tot</t>
+          <t>T</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C15" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D15" t="n">
-        <v>372.3188405797102</v>
+        <v>6.732690320914315</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -883,42 +883,42 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.02063851666184647</v>
+        <v>7.089281163435101e-05</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>NH4+.tot</t>
+          <t>PO4-3.tot</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BB11N</t>
+          <t>BB11Z</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>PP-11N</t>
+          <t>PP-11Z</t>
         </is>
       </c>
       <c r="C16" s="1" t="n">
         <v>45272</v>
       </c>
       <c r="D16" t="n">
-        <v>7.16</v>
+        <v>0.056</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>mg/l</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>7.16</v>
+        <v>1.746180230745245e-06</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>pH</t>
+          <t>S-2.tot</t>
         </is>
       </c>
     </row>

</xml_diff>